<commit_message>
Update TestPlan remove some TestPlan Out
</commit_message>
<xml_diff>
--- a/doc/TestDoc/Test Suite/TestPlanPrincipleCommand.xlsx
+++ b/doc/TestDoc/Test Suite/TestPlanPrincipleCommand.xlsx
@@ -21,9 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="7">
     <font>
       <name val="Aptos Narrow"/>
@@ -329,7 +327,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -452,6 +450,8 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -849,7 +849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="21.77734375" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -991,12 +991,12 @@
     <row r="10">
       <c r="A10" s="39" t="inlineStr">
         <is>
-          <t>ProduceFoodCommand</t>
+          <t>RecruitSoldiersCommand</t>
         </is>
       </c>
       <c r="B10" s="39" t="inlineStr">
         <is>
-          <t>getArmy</t>
+          <t>execute</t>
         </is>
       </c>
       <c r="C10" s="39" t="n">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="B11" s="39" t="inlineStr">
         <is>
-          <t>execute</t>
+          <t>getRecordedAction</t>
         </is>
       </c>
       <c r="C11" s="39" t="n">
@@ -1025,14 +1025,14 @@
       <c r="F11" s="39" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="39" t="inlineStr">
-        <is>
-          <t>RecruitSoldiersCommand</t>
+      <c r="A12" s="47" t="inlineStr">
+        <is>
+          <t>NoneCommand</t>
         </is>
       </c>
       <c r="B12" s="39" t="inlineStr">
         <is>
-          <t>getRecordedAction</t>
+          <t>execute</t>
         </is>
       </c>
       <c r="C12" s="39" t="n">
@@ -1045,12 +1045,12 @@
     <row r="13">
       <c r="A13" s="39" t="inlineStr">
         <is>
-          <t>RecruitSoldiersCommand</t>
+          <t>NoneCommand</t>
         </is>
       </c>
       <c r="B13" s="39" t="inlineStr">
         <is>
-          <t>getArmy</t>
+          <t>getRecordedAction</t>
         </is>
       </c>
       <c r="C13" s="39" t="n">
@@ -1061,18 +1061,18 @@
       <c r="F13" s="39" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="47" t="inlineStr">
-        <is>
-          <t>NoneCommand</t>
+      <c r="A14" s="39" t="inlineStr">
+        <is>
+          <t>CommandFactory</t>
         </is>
       </c>
       <c r="B14" s="39" t="inlineStr">
         <is>
-          <t>execute</t>
+          <t>createCommand</t>
         </is>
       </c>
       <c r="C14" s="39" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D14" s="39" t="n"/>
       <c r="E14" s="39" t="n"/>
@@ -1081,74 +1081,20 @@
     <row r="15">
       <c r="A15" s="39" t="inlineStr">
         <is>
-          <t>NoneCommand</t>
-        </is>
-      </c>
-      <c r="B15" s="39" t="inlineStr">
-        <is>
-          <t>getRecordedAction</t>
-        </is>
-      </c>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B15" s="50" t="n"/>
       <c r="C15" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="39" t="n"/>
-      <c r="E15" s="39" t="n"/>
-      <c r="F15" s="39" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="39" t="inlineStr">
-        <is>
-          <t>NoneCommand</t>
-        </is>
-      </c>
-      <c r="B16" s="39" t="inlineStr">
-        <is>
-          <t>getArmy</t>
-        </is>
-      </c>
-      <c r="C16" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="39" t="n"/>
-      <c r="E16" s="39" t="n"/>
-      <c r="F16" s="39" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="39" t="inlineStr">
-        <is>
-          <t>CommandFactory</t>
-        </is>
-      </c>
-      <c r="B17" s="39" t="inlineStr">
-        <is>
-          <t>createCommand</t>
-        </is>
-      </c>
-      <c r="C17" s="39" t="n">
-        <v>5</v>
-      </c>
-      <c r="D17" s="39" t="n"/>
-      <c r="E17" s="39" t="n"/>
-      <c r="F17" s="39" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="39" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B18" s="41" t="n"/>
-      <c r="C18" s="39" t="n">
-        <v>20</v>
-      </c>
-      <c r="D18" s="41" t="n"/>
-      <c r="E18" s="41" t="n"/>
-      <c r="F18" s="41" t="n"/>
+        <v>17</v>
+      </c>
+      <c r="D15" s="41" t="n"/>
+      <c r="E15" s="41" t="n"/>
+      <c r="F15" s="41" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A15:B15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1170,7 +1116,6 @@
     <col width="8.21875" bestFit="1" customWidth="1" style="2" min="5" max="5"/>
     <col width="13.21875" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
     <col width="34.44140625" bestFit="1" customWidth="1" style="2" min="7" max="7"/>
-    <col width="8.88671875" customWidth="1" style="2" min="8" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1276,7 +1221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:H17"/>
+  <dimension ref="A3:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1286,7 +1231,6 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="3">
@@ -1300,12 +1244,11 @@
           <t>Eternal Crash2</t>
         </is>
       </c>
-      <c r="C3" s="41" t="n"/>
-      <c r="D3" s="41" t="n"/>
-      <c r="E3" s="41" t="n"/>
-      <c r="F3" s="41" t="n"/>
-      <c r="G3" s="41" t="n"/>
-      <c r="H3" s="41" t="n"/>
+      <c r="C3" s="51" t="n"/>
+      <c r="D3" s="51" t="n"/>
+      <c r="E3" s="51" t="n"/>
+      <c r="F3" s="51" t="n"/>
+      <c r="G3" s="50" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="42" t="inlineStr">
@@ -1318,12 +1261,11 @@
           <t>SendArmyCommand</t>
         </is>
       </c>
-      <c r="C4" s="41" t="n"/>
-      <c r="D4" s="41" t="n"/>
-      <c r="E4" s="41" t="n"/>
-      <c r="F4" s="41" t="n"/>
-      <c r="G4" s="41" t="n"/>
-      <c r="H4" s="41" t="n"/>
+      <c r="C4" s="51" t="n"/>
+      <c r="D4" s="51" t="n"/>
+      <c r="E4" s="51" t="n"/>
+      <c r="F4" s="51" t="n"/>
+      <c r="G4" s="50" t="n"/>
     </row>
     <row r="5" ht="35.4" customHeight="1">
       <c r="A5" s="42" t="inlineStr">
@@ -1336,12 +1278,11 @@
           <t>Window 11, java version "1.8.0_503" , Junit 5</t>
         </is>
       </c>
-      <c r="C5" s="41" t="n"/>
-      <c r="D5" s="41" t="n"/>
-      <c r="E5" s="41" t="n"/>
-      <c r="F5" s="41" t="n"/>
-      <c r="G5" s="41" t="n"/>
-      <c r="H5" s="41" t="n"/>
+      <c r="C5" s="51" t="n"/>
+      <c r="D5" s="51" t="n"/>
+      <c r="E5" s="51" t="n"/>
+      <c r="F5" s="51" t="n"/>
+      <c r="G5" s="50" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="42" t="inlineStr">
@@ -1352,12 +1293,11 @@
       <c r="B6" s="45" t="n">
         <v>46305</v>
       </c>
-      <c r="C6" s="41" t="n"/>
-      <c r="D6" s="41" t="n"/>
-      <c r="E6" s="41" t="n"/>
-      <c r="F6" s="41" t="n"/>
-      <c r="G6" s="41" t="n"/>
-      <c r="H6" s="41" t="n"/>
+      <c r="C6" s="51" t="n"/>
+      <c r="D6" s="51" t="n"/>
+      <c r="E6" s="51" t="n"/>
+      <c r="F6" s="51" t="n"/>
+      <c r="G6" s="50" t="n"/>
     </row>
     <row r="7" ht="35.4" customHeight="1">
       <c r="A7" s="42" t="inlineStr">
@@ -1370,12 +1310,11 @@
           <t>Mock ArmyService, GameEventRepository; real City/Player/Game builders</t>
         </is>
       </c>
-      <c r="C7" s="41" t="n"/>
-      <c r="D7" s="41" t="n"/>
-      <c r="E7" s="41" t="n"/>
-      <c r="F7" s="41" t="n"/>
-      <c r="G7" s="41" t="n"/>
-      <c r="H7" s="41" t="n"/>
+      <c r="C7" s="51" t="n"/>
+      <c r="D7" s="51" t="n"/>
+      <c r="E7" s="51" t="n"/>
+      <c r="F7" s="51" t="n"/>
+      <c r="G7" s="50" t="n"/>
     </row>
     <row r="11" ht="21" customHeight="1">
       <c r="A11" s="43" t="inlineStr">
@@ -1438,7 +1377,6 @@
       <c r="E12" s="43" t="n"/>
       <c r="F12" s="43" t="n"/>
       <c r="G12" s="43" t="n"/>
-      <c r="H12" s="48" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="43" t="inlineStr">
@@ -1464,11 +1402,6 @@
       <c r="E13" s="43" t="n"/>
       <c r="F13" s="43" t="n"/>
       <c r="G13" s="43" t="n"/>
-      <c r="H13" s="48" t="inlineStr">
-        <is>
-          <t>SendArmyCommand.java:40-42</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="43" t="inlineStr">
@@ -1494,7 +1427,6 @@
       <c r="E14" s="43" t="n"/>
       <c r="F14" s="43" t="n"/>
       <c r="G14" s="43" t="n"/>
-      <c r="H14" s="48" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="43" t="inlineStr">
@@ -1520,11 +1452,6 @@
       <c r="E15" s="43" t="n"/>
       <c r="F15" s="43" t="n"/>
       <c r="G15" s="43" t="n"/>
-      <c r="H15" s="48" t="inlineStr">
-        <is>
-          <t>SendArmyCommand.java:44-51 - random, needs a seam or a loop assertion</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="43" t="inlineStr">
@@ -1550,11 +1477,6 @@
       <c r="E16" s="43" t="n"/>
       <c r="F16" s="43" t="n"/>
       <c r="G16" s="43" t="n"/>
-      <c r="H16" s="48" t="inlineStr">
-        <is>
-          <t>SendArmyCommand.java:54-60</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="43" t="inlineStr">
@@ -1580,7 +1502,6 @@
       <c r="E17" s="43" t="n"/>
       <c r="F17" s="43" t="n"/>
       <c r="G17" s="43" t="n"/>
-      <c r="H17" s="48" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1600,7 +1521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:H14"/>
+  <dimension ref="A3:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1610,7 +1531,6 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="3">
@@ -1624,12 +1544,11 @@
           <t>Eternal Crash2</t>
         </is>
       </c>
-      <c r="C3" s="41" t="n"/>
-      <c r="D3" s="41" t="n"/>
-      <c r="E3" s="41" t="n"/>
-      <c r="F3" s="41" t="n"/>
-      <c r="G3" s="41" t="n"/>
-      <c r="H3" s="41" t="n"/>
+      <c r="C3" s="51" t="n"/>
+      <c r="D3" s="51" t="n"/>
+      <c r="E3" s="51" t="n"/>
+      <c r="F3" s="51" t="n"/>
+      <c r="G3" s="50" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="44" t="inlineStr">
@@ -1642,12 +1561,11 @@
           <t>ProduceFoodCommand</t>
         </is>
       </c>
-      <c r="C4" s="41" t="n"/>
-      <c r="D4" s="41" t="n"/>
-      <c r="E4" s="41" t="n"/>
-      <c r="F4" s="41" t="n"/>
-      <c r="G4" s="41" t="n"/>
-      <c r="H4" s="41" t="n"/>
+      <c r="C4" s="51" t="n"/>
+      <c r="D4" s="51" t="n"/>
+      <c r="E4" s="51" t="n"/>
+      <c r="F4" s="51" t="n"/>
+      <c r="G4" s="50" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="44" t="inlineStr">
@@ -1660,12 +1578,11 @@
           <t>Window 11, java version "1.8.0_503" , Junit 5</t>
         </is>
       </c>
-      <c r="C5" s="41" t="n"/>
-      <c r="D5" s="41" t="n"/>
-      <c r="E5" s="41" t="n"/>
-      <c r="F5" s="41" t="n"/>
-      <c r="G5" s="41" t="n"/>
-      <c r="H5" s="41" t="n"/>
+      <c r="C5" s="51" t="n"/>
+      <c r="D5" s="51" t="n"/>
+      <c r="E5" s="51" t="n"/>
+      <c r="F5" s="51" t="n"/>
+      <c r="G5" s="50" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="44" t="inlineStr">
@@ -1676,12 +1593,11 @@
       <c r="B6" s="49" t="n">
         <v>46305</v>
       </c>
-      <c r="C6" s="41" t="n"/>
-      <c r="D6" s="41" t="n"/>
-      <c r="E6" s="41" t="n"/>
-      <c r="F6" s="41" t="n"/>
-      <c r="G6" s="41" t="n"/>
-      <c r="H6" s="41" t="n"/>
+      <c r="C6" s="51" t="n"/>
+      <c r="D6" s="51" t="n"/>
+      <c r="E6" s="51" t="n"/>
+      <c r="F6" s="51" t="n"/>
+      <c r="G6" s="50" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="44" t="inlineStr">
@@ -1694,12 +1610,11 @@
           <t>Mock CityService</t>
         </is>
       </c>
-      <c r="C7" s="41" t="n"/>
-      <c r="D7" s="41" t="n"/>
-      <c r="E7" s="41" t="n"/>
-      <c r="F7" s="41" t="n"/>
-      <c r="G7" s="41" t="n"/>
-      <c r="H7" s="41" t="n"/>
+      <c r="C7" s="51" t="n"/>
+      <c r="D7" s="51" t="n"/>
+      <c r="E7" s="51" t="n"/>
+      <c r="F7" s="51" t="n"/>
+      <c r="G7" s="50" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="43" t="inlineStr">
@@ -1762,11 +1677,6 @@
       <c r="E12" s="43" t="n"/>
       <c r="F12" s="43" t="n"/>
       <c r="G12" s="43" t="n"/>
-      <c r="H12" s="48" t="inlineStr">
-        <is>
-          <t>ProduceFoodCommand.java:20</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="43" t="inlineStr">
@@ -1792,33 +1702,6 @@
       <c r="E13" s="43" t="n"/>
       <c r="F13" s="43" t="n"/>
       <c r="G13" s="43" t="n"/>
-      <c r="H13" s="48" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="43" t="inlineStr">
-        <is>
-          <t>TC03</t>
-        </is>
-      </c>
-      <c r="B14" s="43" t="inlineStr">
-        <is>
-          <t>getArmy</t>
-        </is>
-      </c>
-      <c r="C14" s="46" t="inlineStr">
-        <is>
-          <t>any instance</t>
-        </is>
-      </c>
-      <c r="D14" s="46" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="E14" s="43" t="n"/>
-      <c r="F14" s="43" t="n"/>
-      <c r="G14" s="43" t="n"/>
-      <c r="H14" s="48" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1838,7 +1721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:H14"/>
+  <dimension ref="A3:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1848,7 +1731,6 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="3">
@@ -1862,12 +1744,11 @@
           <t>Eternal Crash2</t>
         </is>
       </c>
-      <c r="C3" s="41" t="n"/>
-      <c r="D3" s="41" t="n"/>
-      <c r="E3" s="41" t="n"/>
-      <c r="F3" s="41" t="n"/>
-      <c r="G3" s="41" t="n"/>
-      <c r="H3" s="41" t="n"/>
+      <c r="C3" s="51" t="n"/>
+      <c r="D3" s="51" t="n"/>
+      <c r="E3" s="51" t="n"/>
+      <c r="F3" s="51" t="n"/>
+      <c r="G3" s="50" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="44" t="inlineStr">
@@ -1880,12 +1761,11 @@
           <t>RecruitSoldiersCommand</t>
         </is>
       </c>
-      <c r="C4" s="41" t="n"/>
-      <c r="D4" s="41" t="n"/>
-      <c r="E4" s="41" t="n"/>
-      <c r="F4" s="41" t="n"/>
-      <c r="G4" s="41" t="n"/>
-      <c r="H4" s="41" t="n"/>
+      <c r="C4" s="51" t="n"/>
+      <c r="D4" s="51" t="n"/>
+      <c r="E4" s="51" t="n"/>
+      <c r="F4" s="51" t="n"/>
+      <c r="G4" s="50" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="44" t="inlineStr">
@@ -1898,12 +1778,11 @@
           <t>Window 11, java version "1.8.0_503" , Junit 5</t>
         </is>
       </c>
-      <c r="C5" s="41" t="n"/>
-      <c r="D5" s="41" t="n"/>
-      <c r="E5" s="41" t="n"/>
-      <c r="F5" s="41" t="n"/>
-      <c r="G5" s="41" t="n"/>
-      <c r="H5" s="41" t="n"/>
+      <c r="C5" s="51" t="n"/>
+      <c r="D5" s="51" t="n"/>
+      <c r="E5" s="51" t="n"/>
+      <c r="F5" s="51" t="n"/>
+      <c r="G5" s="50" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="44" t="inlineStr">
@@ -1914,12 +1793,11 @@
       <c r="B6" s="49" t="n">
         <v>46305</v>
       </c>
-      <c r="C6" s="41" t="n"/>
-      <c r="D6" s="41" t="n"/>
-      <c r="E6" s="41" t="n"/>
-      <c r="F6" s="41" t="n"/>
-      <c r="G6" s="41" t="n"/>
-      <c r="H6" s="41" t="n"/>
+      <c r="C6" s="51" t="n"/>
+      <c r="D6" s="51" t="n"/>
+      <c r="E6" s="51" t="n"/>
+      <c r="F6" s="51" t="n"/>
+      <c r="G6" s="50" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="44" t="inlineStr">
@@ -1932,12 +1810,11 @@
           <t>Mock CityService</t>
         </is>
       </c>
-      <c r="C7" s="41" t="n"/>
-      <c r="D7" s="41" t="n"/>
-      <c r="E7" s="41" t="n"/>
-      <c r="F7" s="41" t="n"/>
-      <c r="G7" s="41" t="n"/>
-      <c r="H7" s="41" t="n"/>
+      <c r="C7" s="51" t="n"/>
+      <c r="D7" s="51" t="n"/>
+      <c r="E7" s="51" t="n"/>
+      <c r="F7" s="51" t="n"/>
+      <c r="G7" s="50" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="43" t="inlineStr">
@@ -2000,11 +1877,6 @@
       <c r="E12" s="43" t="n"/>
       <c r="F12" s="43" t="n"/>
       <c r="G12" s="43" t="n"/>
-      <c r="H12" s="48" t="inlineStr">
-        <is>
-          <t>RecruitSoldiersCommand.java:20</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="43" t="inlineStr">
@@ -2030,33 +1902,6 @@
       <c r="E13" s="43" t="n"/>
       <c r="F13" s="43" t="n"/>
       <c r="G13" s="43" t="n"/>
-      <c r="H13" s="48" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="43" t="inlineStr">
-        <is>
-          <t>TC03</t>
-        </is>
-      </c>
-      <c r="B14" s="43" t="inlineStr">
-        <is>
-          <t>getArmy</t>
-        </is>
-      </c>
-      <c r="C14" s="46" t="inlineStr">
-        <is>
-          <t>any instance</t>
-        </is>
-      </c>
-      <c r="D14" s="46" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="E14" s="43" t="n"/>
-      <c r="F14" s="43" t="n"/>
-      <c r="G14" s="43" t="n"/>
-      <c r="H14" s="48" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2076,7 +1921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:H14"/>
+  <dimension ref="A3:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2086,7 +1931,6 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="3">
@@ -2100,12 +1944,11 @@
           <t>Eternal Crash2</t>
         </is>
       </c>
-      <c r="C3" s="41" t="n"/>
-      <c r="D3" s="41" t="n"/>
-      <c r="E3" s="41" t="n"/>
-      <c r="F3" s="41" t="n"/>
-      <c r="G3" s="41" t="n"/>
-      <c r="H3" s="41" t="n"/>
+      <c r="C3" s="51" t="n"/>
+      <c r="D3" s="51" t="n"/>
+      <c r="E3" s="51" t="n"/>
+      <c r="F3" s="51" t="n"/>
+      <c r="G3" s="50" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="44" t="inlineStr">
@@ -2118,12 +1961,11 @@
           <t>NoneCommand</t>
         </is>
       </c>
-      <c r="C4" s="41" t="n"/>
-      <c r="D4" s="41" t="n"/>
-      <c r="E4" s="41" t="n"/>
-      <c r="F4" s="41" t="n"/>
-      <c r="G4" s="41" t="n"/>
-      <c r="H4" s="41" t="n"/>
+      <c r="C4" s="51" t="n"/>
+      <c r="D4" s="51" t="n"/>
+      <c r="E4" s="51" t="n"/>
+      <c r="F4" s="51" t="n"/>
+      <c r="G4" s="50" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="44" t="inlineStr">
@@ -2136,12 +1978,11 @@
           <t>Window 11, java version "1.8.0_503" , Junit 5</t>
         </is>
       </c>
-      <c r="C5" s="41" t="n"/>
-      <c r="D5" s="41" t="n"/>
-      <c r="E5" s="41" t="n"/>
-      <c r="F5" s="41" t="n"/>
-      <c r="G5" s="41" t="n"/>
-      <c r="H5" s="41" t="n"/>
+      <c r="C5" s="51" t="n"/>
+      <c r="D5" s="51" t="n"/>
+      <c r="E5" s="51" t="n"/>
+      <c r="F5" s="51" t="n"/>
+      <c r="G5" s="50" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="44" t="inlineStr">
@@ -2152,12 +1993,11 @@
       <c r="B6" s="49" t="n">
         <v>46305</v>
       </c>
-      <c r="C6" s="41" t="n"/>
-      <c r="D6" s="41" t="n"/>
-      <c r="E6" s="41" t="n"/>
-      <c r="F6" s="41" t="n"/>
-      <c r="G6" s="41" t="n"/>
-      <c r="H6" s="41" t="n"/>
+      <c r="C6" s="51" t="n"/>
+      <c r="D6" s="51" t="n"/>
+      <c r="E6" s="51" t="n"/>
+      <c r="F6" s="51" t="n"/>
+      <c r="G6" s="50" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="44" t="inlineStr">
@@ -2170,12 +2010,11 @@
           <t>None (no dependencies)</t>
         </is>
       </c>
-      <c r="C7" s="41" t="n"/>
-      <c r="D7" s="41" t="n"/>
-      <c r="E7" s="41" t="n"/>
-      <c r="F7" s="41" t="n"/>
-      <c r="G7" s="41" t="n"/>
-      <c r="H7" s="41" t="n"/>
+      <c r="C7" s="51" t="n"/>
+      <c r="D7" s="51" t="n"/>
+      <c r="E7" s="51" t="n"/>
+      <c r="F7" s="51" t="n"/>
+      <c r="G7" s="50" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="43" t="inlineStr">
@@ -2238,11 +2077,6 @@
       <c r="E12" s="43" t="n"/>
       <c r="F12" s="43" t="n"/>
       <c r="G12" s="43" t="n"/>
-      <c r="H12" s="48" t="inlineStr">
-        <is>
-          <t>NoneCommand.java:8</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="43" t="inlineStr">
@@ -2268,33 +2102,6 @@
       <c r="E13" s="43" t="n"/>
       <c r="F13" s="43" t="n"/>
       <c r="G13" s="43" t="n"/>
-      <c r="H13" s="48" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="43" t="inlineStr">
-        <is>
-          <t>TC03</t>
-        </is>
-      </c>
-      <c r="B14" s="43" t="inlineStr">
-        <is>
-          <t>getArmy</t>
-        </is>
-      </c>
-      <c r="C14" s="46" t="inlineStr">
-        <is>
-          <t>any instance</t>
-        </is>
-      </c>
-      <c r="D14" s="46" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="E14" s="43" t="n"/>
-      <c r="F14" s="43" t="n"/>
-      <c r="G14" s="43" t="n"/>
-      <c r="H14" s="48" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2314,7 +2121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:H16"/>
+  <dimension ref="A3:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2324,7 +2131,6 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="3">
@@ -2338,12 +2144,11 @@
           <t>Eternal Crash2</t>
         </is>
       </c>
-      <c r="C3" s="41" t="n"/>
-      <c r="D3" s="41" t="n"/>
-      <c r="E3" s="41" t="n"/>
-      <c r="F3" s="41" t="n"/>
-      <c r="G3" s="41" t="n"/>
-      <c r="H3" s="41" t="n"/>
+      <c r="C3" s="51" t="n"/>
+      <c r="D3" s="51" t="n"/>
+      <c r="E3" s="51" t="n"/>
+      <c r="F3" s="51" t="n"/>
+      <c r="G3" s="50" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="44" t="inlineStr">
@@ -2356,12 +2161,11 @@
           <t>CommandFactory</t>
         </is>
       </c>
-      <c r="C4" s="41" t="n"/>
-      <c r="D4" s="41" t="n"/>
-      <c r="E4" s="41" t="n"/>
-      <c r="F4" s="41" t="n"/>
-      <c r="G4" s="41" t="n"/>
-      <c r="H4" s="41" t="n"/>
+      <c r="C4" s="51" t="n"/>
+      <c r="D4" s="51" t="n"/>
+      <c r="E4" s="51" t="n"/>
+      <c r="F4" s="51" t="n"/>
+      <c r="G4" s="50" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="44" t="inlineStr">
@@ -2374,12 +2178,11 @@
           <t>Window 11, java version "1.8.0_503" , Junit 5</t>
         </is>
       </c>
-      <c r="C5" s="41" t="n"/>
-      <c r="D5" s="41" t="n"/>
-      <c r="E5" s="41" t="n"/>
-      <c r="F5" s="41" t="n"/>
-      <c r="G5" s="41" t="n"/>
-      <c r="H5" s="41" t="n"/>
+      <c r="C5" s="51" t="n"/>
+      <c r="D5" s="51" t="n"/>
+      <c r="E5" s="51" t="n"/>
+      <c r="F5" s="51" t="n"/>
+      <c r="G5" s="50" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="44" t="inlineStr">
@@ -2390,12 +2193,11 @@
       <c r="B6" s="49" t="n">
         <v>46305</v>
       </c>
-      <c r="C6" s="41" t="n"/>
-      <c r="D6" s="41" t="n"/>
-      <c r="E6" s="41" t="n"/>
-      <c r="F6" s="41" t="n"/>
-      <c r="G6" s="41" t="n"/>
-      <c r="H6" s="41" t="n"/>
+      <c r="C6" s="51" t="n"/>
+      <c r="D6" s="51" t="n"/>
+      <c r="E6" s="51" t="n"/>
+      <c r="F6" s="51" t="n"/>
+      <c r="G6" s="50" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="44" t="inlineStr">
@@ -2408,12 +2210,11 @@
           <t>Mock CityService, ArmyService, GameEventRepository; real City/Game</t>
         </is>
       </c>
-      <c r="C7" s="41" t="n"/>
-      <c r="D7" s="41" t="n"/>
-      <c r="E7" s="41" t="n"/>
-      <c r="F7" s="41" t="n"/>
-      <c r="G7" s="41" t="n"/>
-      <c r="H7" s="41" t="n"/>
+      <c r="C7" s="51" t="n"/>
+      <c r="D7" s="51" t="n"/>
+      <c r="E7" s="51" t="n"/>
+      <c r="F7" s="51" t="n"/>
+      <c r="G7" s="50" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="43" t="inlineStr">
@@ -2476,11 +2277,6 @@
       <c r="E12" s="43" t="n"/>
       <c r="F12" s="43" t="n"/>
       <c r="G12" s="43" t="n"/>
-      <c r="H12" s="48" t="inlineStr">
-        <is>
-          <t>CommandFactory.java:23</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="43" t="inlineStr">
@@ -2506,11 +2302,6 @@
       <c r="E13" s="43" t="n"/>
       <c r="F13" s="43" t="n"/>
       <c r="G13" s="43" t="n"/>
-      <c r="H13" s="48" t="inlineStr">
-        <is>
-          <t>CommandFactory.java:24</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="43" t="inlineStr">
@@ -2536,11 +2327,6 @@
       <c r="E14" s="43" t="n"/>
       <c r="F14" s="43" t="n"/>
       <c r="G14" s="43" t="n"/>
-      <c r="H14" s="48" t="inlineStr">
-        <is>
-          <t>CommandFactory.java:25</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="43" t="inlineStr">
@@ -2566,11 +2352,6 @@
       <c r="E15" s="43" t="n"/>
       <c r="F15" s="43" t="n"/>
       <c r="G15" s="43" t="n"/>
-      <c r="H15" s="48" t="inlineStr">
-        <is>
-          <t>CommandFactory.java:26</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="43" t="inlineStr">
@@ -2596,11 +2377,6 @@
       <c r="E16" s="43" t="n"/>
       <c r="F16" s="43" t="n"/>
       <c r="G16" s="43" t="n"/>
-      <c r="H16" s="48" t="inlineStr">
-        <is>
-          <t>CommandFactory.java:20</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>